<commit_message>
Add home, transfers, news, services and about UI specs, update docs
</commit_message>
<xml_diff>
--- a/docs/Final_Project_UI_Bug_Siyahisi.xlsx
+++ b/docs/Final_Project_UI_Bug_Siyahisi.xlsx
@@ -864,7 +864,7 @@
     <t xml:space="preserve">Avtomatlaşdırma</t>
   </si>
   <si>
-    <t xml:space="preserve">65 Selenium ssenarisi: 43 sabit, 22 məlum bug (known-bug) ssenarisi</t>
+    <t xml:space="preserve">97 Selenium ssenarisi: 75 sabit (hamısı keçir), 22 məlum bug (known-bug) ssenarisi</t>
   </si>
   <si>
     <t xml:space="preserve">Screenshot</t>
@@ -1153,9 +1153,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>183240</xdr:colOff>
+      <xdr:colOff>182880</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>17640</xdr:rowOff>
+      <xdr:rowOff>17280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1169,7 +1169,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="571680"/>
-          <a:ext cx="10476000" cy="6303960"/>
+          <a:ext cx="10475640" cy="6303600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1190,9 +1190,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>183240</xdr:colOff>
+      <xdr:colOff>182880</xdr:colOff>
       <xdr:row>73</xdr:row>
-      <xdr:rowOff>17640</xdr:rowOff>
+      <xdr:rowOff>17280</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1206,7 +1206,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="7620120"/>
-          <a:ext cx="10476000" cy="6303960"/>
+          <a:ext cx="10475640" cy="6303600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Update UI test results and bug list
</commit_message>
<xml_diff>
--- a/docs/Final_Project_UI_Bug_Siyahisi.xlsx
+++ b/docs/Final_Project_UI_Bug_Siyahisi.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="308">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -831,6 +831,113 @@
     <t xml:space="preserve">Selenium diaqnostikasında müşahidə olunub; əl ilə sildikdə də təkrarlanıb-təkrarlanmadığı yoxlanmalıdır</t>
   </si>
   <si>
+    <t xml:space="preserve">BUG-024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Məbləğ sahəsi maksimum limiti (80 000) yoxlamır</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. /az açın
+2. Kalkulyatorda məbləğ sahəsinə 99999999 yazın</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limit xətası və ya dəyərin 80 000-ə məhdudlaşdırılması</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sahə 99999999 qəbul edir, slayder 80000-də qalır (sinxron deyil), cəmi 101 822 141.21 AZN göstərilir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brauzerdə əl ilə təsdiqləndi (UI-CAL-018)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ana səhifə</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Konsolda resurs və CORS xətaları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. /az açın
+2. Brauzer konsoluna baxın</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xəta yoxdur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORS (infobank.az), 404, 400, ERR_TOO_MANY_REDIRECTS və timeout xətaları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bəzi timeout-lar test mühitindən ola bilər (UI-HOM-005)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUG-026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Əmanətlər</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Əmanət kalkulyatoru minimum məbləğdən (100) az dəyəri qəbul edir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. /az/emanetler/digital-depozit açın
+2. Məbləğ sahəsinə 99 yazın</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xəta mesajı və ya rədd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">99 qəbul edilir, 99.60 AZN cəmi göstərilir, xəta yoxdur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brauzerdə əl ilə təsdiqləndi (UI-DEP-018)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBS-015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kampaniyalar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vaxtı bitmiş müsabiqə hələ də siyahıdadır</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. /az/kampaniyalar açın
+2. "İstanbula 2 nəfərlik bilet" kampaniyasına baxın</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bitmiş kampaniya aktiv kimi görünmür</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Müsabiqə 17–27 iyul 2026 üçün idi, oktyabrda hələ siyahıdadır</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biznes ilə dəqiqləşdirmək (UI-CMP-002)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBS-016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEO və dillər</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/en və /ru səhifələrində html lang="az", başlıq AZ; daxili səhifələrdə canonical /az-a işarə edir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. /en və /ru açın, html lang və title-a baxın
+2. /az/kartlar/debet canonical-a baxın</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lang="en"/"ru", müvafiq başlıq; canonical öz URL-ni göstərir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lang="az" və AZ başlıq; canonical https://www.bankofbaku.com/az; /az/biznes başlığı ana səhifə başlığıdır</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UI-LNG-003, 004, ERR-002, BIZ-002</t>
+  </si>
+  <si>
     <t xml:space="preserve">Say</t>
   </si>
   <si>
@@ -852,13 +959,13 @@
     <t xml:space="preserve">Qalan yoxlamalar</t>
   </si>
   <si>
-    <t xml:space="preserve">Rəng kontrastı, klaviatura fokusu, yüklənmə müddəti, valyuta (USD/EUR) əmanət hesablaması, FAQ akkordeonu</t>
+    <t xml:space="preserve">Qalan 21 case: hücum xarakterli (ERR-003, SRC-004, SEC-005), offline (ERR-004), kontrast/fokus (A11-002, 005), performans (PRF-001), dil qaydaları (LNG-005…012), NAV-013, HOM-002, CAL-017, 019, 020, CHT-004</t>
   </si>
   <si>
     <t xml:space="preserve">Bug-ların biznesə təqdimi</t>
   </si>
   <si>
-    <t xml:space="preserve">BUG-017 – 023 və OBS-006 – 014 üçün biznes təsdiqi lazımdır</t>
+    <t xml:space="preserve">BUG-017 – 026 və OBS-006 – 016 üçün biznes təsdiqi lazımdır</t>
   </si>
   <si>
     <t xml:space="preserve">Avtomatlaşdırma</t>
@@ -1153,9 +1260,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>182880</xdr:colOff>
+      <xdr:colOff>182160</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>17280</xdr:rowOff>
+      <xdr:rowOff>16560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1169,7 +1276,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="571680"/>
-          <a:ext cx="10475640" cy="6303600"/>
+          <a:ext cx="10474920" cy="6302880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1190,9 +1297,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>182880</xdr:colOff>
+      <xdr:colOff>182160</xdr:colOff>
       <xdr:row>73</xdr:row>
-      <xdr:rowOff>17280</xdr:rowOff>
+      <xdr:rowOff>16560</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1206,7 +1313,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="7620120"/>
-          <a:ext cx="10475640" cy="6303600"/>
+          <a:ext cx="10474920" cy="6302880"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1401,7 +1508,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
@@ -2515,6 +2622,151 @@
       </c>
       <c r="I38" s="3" t="s">
         <v>256</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -2556,7 +2808,7 @@
         <v>6</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>257</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2574,7 +2826,7 @@
       </c>
       <c r="B3" s="5" t="n">
         <f aca="false">COUNTIFS('Bug siyahısı'!G2:G200,A3,'Bug siyahısı'!H2:H200,"&lt;&gt;Rədd edildi")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2583,16 +2835,16 @@
       </c>
       <c r="B4" s="5" t="n">
         <f aca="false">COUNTIFS('Bug siyahısı'!G2:G200,A4,'Bug siyahısı'!H2:H200,"&lt;&gt;Rədd edildi")</f>
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>258</v>
+        <v>292</v>
       </c>
       <c r="B5" s="6" t="n">
         <f aca="false">SUM(B2:B4)</f>
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2621,10 +2873,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>259</v>
+        <v>293</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>260</v>
+        <v>294</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>8</v>
@@ -2635,10 +2887,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>261</v>
+        <v>295</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>262</v>
+        <v>296</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2646,10 +2898,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>263</v>
+        <v>297</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>264</v>
+        <v>298</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2657,10 +2909,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>265</v>
+        <v>299</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>266</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2668,10 +2920,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>267</v>
+        <v>301</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>268</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2679,10 +2931,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>269</v>
+        <v>303</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>270</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>
@@ -2711,17 +2963,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>271</v>
+        <v>305</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>272</v>
+        <v>306</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>273</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalize UI docs and bug list
</commit_message>
<xml_diff>
--- a/docs/Final_Project_UI_Bug_Siyahisi.xlsx
+++ b/docs/Final_Project_UI_Bug_Siyahisi.xlsx
@@ -204,7 +204,7 @@
     <t xml:space="preserve">Dil</t>
   </si>
   <si>
-    <t xml:space="preserve">/en səhifəsində html lang atributu "az" qalır</t>
+    <t xml:space="preserve">/en və /ru səhifələrində html lang atributu "az" qalır</t>
   </si>
   <si>
     <t xml:space="preserve">1. https://www.bankofbaku.com/en açın
@@ -217,13 +217,13 @@
     <t xml:space="preserve">lang="az"</t>
   </si>
   <si>
-    <t xml:space="preserve">Ekran oxuyucular və SEO üçün səhv dil; avtomatik test ilə təsdiqləndi</t>
+    <t xml:space="preserve">Ekran oxuyucular və SEO üçün səhv dil; avtomatik test ilə təsdiqləndi; /ru üçün də 12.10.2026 əl ilə təsdiqləndi</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-009</t>
   </si>
   <si>
-    <t xml:space="preserve">/en səhifəsinin başlığı (title) Azərbaycan dilindədir</t>
+    <t xml:space="preserve">/en və /ru səhifələrinin başlığı (title) Azərbaycan dilindədir</t>
   </si>
   <si>
     <t xml:space="preserve">1. /en açın
@@ -236,7 +236,7 @@
     <t xml:space="preserve">"Bank of Baku - Sizə yaxın bankçılıq!"</t>
   </si>
   <si>
-    <t xml:space="preserve">SEO və istifadəçi təcrübəsi; avtomatik test ilə təsdiqləndi</t>
+    <t xml:space="preserve">SEO və istifadəçi təcrübəsi; avtomatik test ilə təsdiqləndi; /ru üçün də 12.10.2026 əl ilə təsdiqləndi</t>
   </si>
   <si>
     <t xml:space="preserve">BUG-010</t>
@@ -683,20 +683,20 @@
     <t xml:space="preserve">SEO və dillər</t>
   </si>
   <si>
-    <t xml:space="preserve">/en və /ru səhifələrində html lang="az", başlıq AZ; daxili səhifələrdə canonical /az-a işarə edir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. /en və /ru açın, html lang və title-a baxın
-2. /az/kartlar/debet canonical-a baxın</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lang="en"/"ru", müvafiq başlıq; canonical öz URL-ni göstərir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lang="az" və AZ başlıq; canonical https://www.bankofbaku.com/az; /az/biznes başlığı ana səhifə başlığıdır</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UI-LNG-003, 004, ERR-002, BIZ-002</t>
+    <t xml:space="preserve">Daxili səhifələrdə canonical linki həmişə /az ana səhifəsinə işarə edir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. /az/kartlar/debet açın
+2. Səhifə mənbəyində &lt;link rel="canonical"&gt; dəyərinə baxın</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Canonical səhifənin öz ünvanını göstərməlidir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">canonical = https://www.bankofbaku.com/az (daxili səhifə üçün də)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axtarış sistemləri daxili səhifələri ana səhifənin təkrarı kimi görə bilər (UI-ERR-002)</t>
   </si>
   <si>
     <t xml:space="preserve">Say</t>
@@ -1021,9 +1021,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>181080</xdr:colOff>
+      <xdr:colOff>180720</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>15480</xdr:rowOff>
+      <xdr:rowOff>15120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1037,7 +1037,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="571680"/>
-          <a:ext cx="10473840" cy="6301800"/>
+          <a:ext cx="10473480" cy="6301440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1058,9 +1058,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>181080</xdr:colOff>
+      <xdr:colOff>180720</xdr:colOff>
       <xdr:row>73</xdr:row>
-      <xdr:rowOff>15480</xdr:rowOff>
+      <xdr:rowOff>15120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1074,7 +1074,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="7620120"/>
-          <a:ext cx="10473840" cy="6301800"/>
+          <a:ext cx="10473480" cy="6301440"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>